<commit_message>
align to right for amount & quantity
</commit_message>
<xml_diff>
--- a/portlets/NGeP-portlet/docroot/WEB-INF/templates/ct/loaContent/jadual-harga.xlsx
+++ b/portlets/NGeP-portlet/docroot/WEB-INF/templates/ct/loaContent/jadual-harga.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="60" windowWidth="20115" windowHeight="8010" activeTab="1"/>
@@ -102,12 +102,24 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -415,10 +427,10 @@
     <col min="1" max="1" width="5.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="5.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="5.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.5703125" style="6" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20" style="6" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -431,16 +443,16 @@
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="5" t="s">
         <v>6</v>
       </c>
     </row>
@@ -458,13 +470,13 @@
     <col min="1" max="1" width="4.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="4.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="7.85546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="27.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.7109375" style="6" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="27.42578125" style="6" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -477,25 +489,25 @@
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="5" t="s">
         <v>11</v>
       </c>
     </row>

</xml_diff>

<commit_message>
add tier column for productSheet
</commit_message>
<xml_diff>
--- a/portlets/NGeP-portlet/docroot/WEB-INF/templates/ct/loaContent/jadual-harga.xlsx
+++ b/portlets/NGeP-portlet/docroot/WEB-INF/templates/ct/loaContent/jadual-harga.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="60" windowWidth="20115" windowHeight="8010" activeTab="1"/>
+    <workbookView xWindow="240" yWindow="60" windowWidth="20115" windowHeight="8010"/>
   </bookViews>
   <sheets>
     <sheet name="ProductSheet" sheetId="1" r:id="rId1"/>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="13">
   <si>
     <t>Item</t>
   </si>
@@ -51,6 +51,9 @@
   </si>
   <si>
     <t>Total Amount (No. of Years )(RM)</t>
+  </si>
+  <si>
+    <t>Tier</t>
   </si>
 </sst>
 </file>
@@ -102,7 +105,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -115,10 +118,13 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -421,19 +427,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="5.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="5.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16" style="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.5703125" style="6" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20" style="6" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.85546875" style="6" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16" style="6" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.5703125" style="7" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20" style="7" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>3</v>
       </c>
@@ -443,16 +450,19 @@
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="5" t="s">
+      <c r="G1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="H1" s="5" t="s">
         <v>6</v>
       </c>
     </row>
@@ -474,9 +484,9 @@
     <col min="5" max="5" width="14.5703125" style="4" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="17.28515625" style="4" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="15.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="7.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.7109375" style="6" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="27.42578125" style="6" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.85546875" style="6" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.7109375" style="7" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="27.42578125" style="7" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -501,7 +511,7 @@
       <c r="G1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="I1" s="5" t="s">

</xml_diff>